<commit_message>
set up dbever prisma
</commit_message>
<xml_diff>
--- a/catatan/catatan install prisma .xlsx
+++ b/catatan/catatan install prisma .xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="22188" windowHeight="8400"/>
+    <workbookView windowWidth="22188" windowHeight="9000"/>
   </bookViews>
   <sheets>
     <sheet name="catatan install prisma " sheetId="1" r:id="rId1"/>
@@ -32,13 +32,13 @@
     <t xml:space="preserve">instalasi prisma </t>
   </si>
   <si>
-    <t>npm install prisma@7@pridma/client@7</t>
+    <t>npm install prisma@7 @prisma/client@7</t>
   </si>
   <si>
     <t>npx prisma --version</t>
   </si>
   <si>
-    <t>npm install prisma/adapter-mariadb mariadb</t>
+    <t>npm install @prisma/adapter-mariadb mariadb</t>
   </si>
   <si>
     <t>npx prisma init</t>

</xml_diff>